<commit_message>
IAT source jumper on every motherboard; wideband MCU flashed through the main MCU
- motherboards (1989-93 / 1994-95 rev 0.5, 1996-97 / 1999-2000 / 2001-05
  rev 0.3): the R4/R5 0R links are replaced by JP1, a 1x3 2.54 mm header with
  a removable shunt (STOCK = harness sensor, EXT = IAT connector, default)
- daughterboard rev 0.4: USART3 (PD8/PD9) to the STM32F042's ROM-bootloader
  USART1 (PA9/PA10), plus PD10 -> its BOOT0 and PD11 -> its NRST, so both
  MCUs can be flashed over the one USB-C port (rusEFI support to be written;
  SWD pads kept as a fallback)
- scripts: schematic check now also catches nets split across sheets;
  motherboard project template bundled
- README: flashing and IAT sections

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012UFcA8PhPqkqYxcgEjD2n9
</commit_message>
<xml_diff>
--- a/daughterboard/miata_ecu_daughterboard_parts.xlsx
+++ b/daughterboard/miata_ecu_daughterboard_parts.xlsx
@@ -6592,7 +6592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7109,399 +7109,463 @@
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>PD12</t>
+          <t>PD8</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>LED_RUN</t>
+          <t>WB_PROG_TX</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>PD13</t>
+          <t>PD9</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>LED_COMM</t>
+          <t>WB_PROG_RX</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>PD14</t>
+          <t>PD10</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>LED_WARN</t>
+          <t>WB_BOOT0</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>PD15</t>
+          <t>PD11</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>LED_ERR</t>
+          <t>WB_NRST</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>PC6</t>
+          <t>PD12</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>UART_TX</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>USART3 TX (3.3V, Bluetooth etc.)</t>
-        </is>
-      </c>
+          <t>LED_RUN</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>PC7</t>
+          <t>PD13</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>UART_RX</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>USART3 RX</t>
-        </is>
-      </c>
+          <t>LED_COMM</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>PA11</t>
+          <t>PD14</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>USB_DM</t>
-        </is>
-      </c>
-      <c r="D38" s="10" t="inlineStr">
-        <is>
-          <t>USB D- to motherboard USB-C</t>
-        </is>
-      </c>
+          <t>LED_WARN</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>PA12</t>
+          <t>PD15</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>USB_DP</t>
-        </is>
-      </c>
-      <c r="D39" s="10" t="inlineStr">
-        <is>
-          <t>USB D+</t>
-        </is>
-      </c>
+          <t>LED_ERR</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>PA13</t>
+          <t>PC6</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>SWDIO</t>
+          <t>UART_TX</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>SWD data</t>
+          <t>USART3 TX (3.3V, Bluetooth etc.)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>PA14</t>
+          <t>PC7</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>SWCLK</t>
+          <t>UART_RX</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>SWD clock</t>
+          <t>USART3 RX</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>PD5</t>
+          <t>PA11</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>ALT_CTL</t>
-        </is>
-      </c>
-      <c r="D42" s="10" t="inlineStr"/>
+          <t>USB_DM</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>USB D- to motherboard USB-C</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>PD6</t>
+          <t>PA12</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>BOOST_CTL</t>
-        </is>
-      </c>
-      <c r="D43" s="10" t="inlineStr"/>
+          <t>USB_DP</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>USB D+</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>PD7</t>
+          <t>PA13</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>VVT_CTL</t>
-        </is>
-      </c>
-      <c r="D44" s="10" t="inlineStr"/>
+          <t>SWDIO</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>SWD data</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>PB3</t>
+          <t>PA14</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>IACV_CTL</t>
-        </is>
-      </c>
-      <c r="D45" s="10" t="inlineStr"/>
+          <t>SWCLK</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>SWD clock</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PD5</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>INJ4_CTL</t>
+          <t>ALT_CTL</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>PB5</t>
+          <t>PD6</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>INJ3_CTL</t>
+          <t>BOOST_CTL</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>PB6</t>
+          <t>PD7</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>INJ2_CTL</t>
+          <t>VVT_CTL</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>PB7</t>
+          <t>PB3</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>INJ1_CTL</t>
+          <t>IACV_CTL</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>BOOT0</t>
+          <t>PB4</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>BOOT0</t>
-        </is>
-      </c>
-      <c r="D50" s="10" t="inlineStr">
-        <is>
-          <t>DFU boot select</t>
-        </is>
-      </c>
+          <t>INJ4_CTL</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>PB8</t>
+          <t>PB5</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>IGN4_CTL</t>
+          <t>INJ3_CTL</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>PB9</t>
+          <t>PB6</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>IGN3_CTL</t>
+          <t>INJ2_CTL</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>PE0</t>
+          <t>PB7</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>IGN2_CTL</t>
+          <t>INJ1_CTL</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n">
+        <v>94</v>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>BOOT0</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>BOOT0</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>DFU boot select</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>PB8</t>
+        </is>
+      </c>
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>IGN4_CTL</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="n">
+        <v>96</v>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>PB9</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>IGN3_CTL</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="n">
+        <v>97</v>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>PE0</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>IGN2_CTL</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="n">
         <v>98</v>
       </c>
-      <c r="B54" s="10" t="inlineStr">
+      <c r="B58" s="10" t="inlineStr">
         <is>
           <t>PE1</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
+      <c r="C58" s="10" t="inlineStr">
         <is>
           <t>IGN1_CTL</t>
         </is>
       </c>
-      <c r="D54" s="10" t="inlineStr"/>
+      <c r="D58" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daughterboard: 5.5 A buck inductor, 33 pF crystal caps; NB alternator control off by default
- L2: Sunlord MWSA0603S-100MT (C132141, 10 uH, Isat 5.5 A, 7 x 6.6 mm). The
  MWSA0503S saturated at 3.5 A, below the LMR14020's 3.8 A maximum current
  limit. Placed on end; D9 and the feedback divider moved 0.3 mm left.
- C13/C14: 33 pF C0G (C1663) for the 20 pF crystal (were 22 pF).
- Firmware: NB alternator control ships off until the field current is
  measured (pin, PID and target still set up). Test checks the field isn't
  driven with the default tune.
- Daughterboard re-routed and released: 754 pads match, 0 unconnected,
  0 clearance errors. Viewer assets and README renders refreshed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012UFcA8PhPqkqYxcgEjD2n9
</commit_message>
<xml_diff>
--- a/daughterboard/miata_ecu_daughterboard_parts.xlsx
+++ b/daughterboard/miata_ecu_daughterboard_parts.xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>22p</t>
+          <t>33p</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr"/>
@@ -819,12 +819,12 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>C1653</t>
+          <t>C1663</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
@@ -835,7 +835,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>CL10C220JB8NNNC</t>
+          <t>CL10C330JB8NNNC</t>
         </is>
       </c>
     </row>
@@ -1788,12 +1788,12 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>L_Sunlord_MWSA0503S</t>
+          <t>L_Sunlord_MWSA0603S</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>C139506</t>
+          <t>C132141</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>MWSA0503-100MT</t>
+          <t>MWSA0603S-100MT</t>
         </is>
       </c>
     </row>
@@ -2433,8 +2433,16 @@
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr"/>
-      <c r="J43" s="4" t="inlineStr"/>
-      <c r="K43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>SS36(SMA)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -3781,8 +3789,16 @@
         </is>
       </c>
       <c r="I75" s="5" t="inlineStr"/>
-      <c r="J75" s="4" t="inlineStr"/>
-      <c r="K75" s="4" t="inlineStr"/>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>JSCJ</t>
+        </is>
+      </c>
+      <c r="K75" s="4" t="inlineStr">
+        <is>
+          <t>1N4148WS</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -5512,8 +5528,16 @@
         </is>
       </c>
       <c r="I114" s="5" t="inlineStr"/>
-      <c r="J114" s="4" t="inlineStr"/>
-      <c r="K114" s="4" t="inlineStr"/>
+      <c r="J114" s="4" t="inlineStr">
+        <is>
+          <t>BOURNS</t>
+        </is>
+      </c>
+      <c r="K114" s="4" t="inlineStr">
+        <is>
+          <t>SMAJ33A</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -5551,8 +5575,16 @@
         </is>
       </c>
       <c r="I115" s="5" t="inlineStr"/>
-      <c r="J115" s="4" t="inlineStr"/>
-      <c r="K115" s="4" t="inlineStr"/>
+      <c r="J115" s="4" t="inlineStr">
+        <is>
+          <t>PTTC(Polytronics Tech)</t>
+        </is>
+      </c>
+      <c r="K115" s="4" t="inlineStr">
+        <is>
+          <t>SMD1206P050TF/24</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
@@ -5641,8 +5673,16 @@
         </is>
       </c>
       <c r="I117" s="5" t="inlineStr"/>
-      <c r="J117" s="4" t="inlineStr"/>
-      <c r="K117" s="4" t="inlineStr"/>
+      <c r="J117" s="4" t="inlineStr">
+        <is>
+          <t>Texas Instruments</t>
+        </is>
+      </c>
+      <c r="K117" s="4" t="inlineStr">
+        <is>
+          <t>SN74LVC4245APWR</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">

</xml_diff>